<commit_message>
Resultados de testes manuais e observações
</commit_message>
<xml_diff>
--- a/tests/Plano_Testes.xlsx
+++ b/tests/Plano_Testes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\My Drive\UNI\2025\2025-2Sem\LDS - Lab Dev Soft\Dev\main\stock-manager\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{527247C9-F7E6-4BAA-8D38-62542F4C1562}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2350A951-4B30-40EF-A268-12ADACAD7FBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0A75782E-02F7-4F60-908F-84060434E598}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="358">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="677" uniqueCount="371">
   <si>
     <t>Plano de testes</t>
   </si>
@@ -656,18 +656,6 @@
     <t>Testes Unitários Dinâmicos – Caixa Aberta</t>
   </si>
   <si>
-    <t>MU5</t>
-  </si>
-  <si>
-    <t>Remoção com stock insuficiente</t>
-  </si>
-  <si>
-    <t>Quantidade superior ao stock</t>
-  </si>
-  <si>
-    <t>Estado interno mantém-se inalterado</t>
-  </si>
-  <si>
     <t>MU6</t>
   </si>
   <si>
@@ -968,18 +956,6 @@
     <t>Resultados apresentados corretamente pela View em cada fluxo, sem erros de navegação</t>
   </si>
   <si>
-    <t>CI7</t>
-  </si>
-  <si>
-    <t>Sequência de operações</t>
-  </si>
-  <si>
-    <t>Várias ações seguidas</t>
-  </si>
-  <si>
-    <t>Estado consistente</t>
-  </si>
-  <si>
     <t>GIG1</t>
   </si>
   <si>
@@ -1113,6 +1089,69 @@
   </si>
   <si>
     <t>A aplicação continua estável, sem degradação visível, sem crash e sem duplicação anómala do menu</t>
+  </si>
+  <si>
+    <t>Confirmado: quando o Model sinaliza stock insuficiente, a View apresenta "✖ Stock insuficiente." e a aplicação continua a correr.</t>
+  </si>
+  <si>
+    <t>7;11;44;46</t>
+  </si>
+  <si>
+    <t>Confirmado: com lista vazia, a View apresenta "--- STOCK ---" e "Sem produtos." sem erro.</t>
+  </si>
+  <si>
+    <t>7;44;53</t>
+  </si>
+  <si>
+    <t>Confirmado: MostrarStock apenas percorre a lista recebida e apresenta os produtos, sem alterar os dados.</t>
+  </si>
+  <si>
+    <t>7;44</t>
+  </si>
+  <si>
+    <t>Confirmado: após CarregarDados(), o fluxo Controller -&gt; View apresenta os produtos no formato "Nome - Quantidade Unidade (mín: QuantidadeMinima)".</t>
+  </si>
+  <si>
+    <t>26;27;44</t>
+  </si>
+  <si>
+    <t>Confirmado: os fluxos de consulta, adição, remoção, reposição e saída têm apresentação coerente na View e não mostram erros de navegação.</t>
+  </si>
+  <si>
+    <t>Confirmado: com stock suficiente, o Model decrementa a quantidade, guarda os dados e a View apresenta confirmação de remoção.</t>
+  </si>
+  <si>
+    <t>25;48</t>
+  </si>
+  <si>
+    <t>Confirmado: com stock insuficiente, o Model não altera os dados, sinaliza erro e a aplicação continua sem crash.</t>
+  </si>
+  <si>
+    <t>46;48</t>
+  </si>
+  <si>
+    <t>Confirmado: os produtos com Quantidade &lt; QuantidadeMinima são filtrados pelo Model e apresentados correctamente pela View.</t>
+  </si>
+  <si>
+    <t>24;48</t>
+  </si>
+  <si>
+    <t>Confirmado: após registo e remoção, GuardarDados() persiste o estado; num reinício, CarregarDados() repõe esse estado.</t>
+  </si>
+  <si>
+    <t>26;51;55</t>
+  </si>
+  <si>
+    <t>Confirmado: quando a remoção falha, o Model termina sem alterar a quantidade e a consulta posterior devolve o estado anterior.</t>
+  </si>
+  <si>
+    <t>25;46</t>
+  </si>
+  <si>
+    <t>Confirmado: opções inválidas repetidas apenas geram mensagem de erro, mantendo o ciclo principal estável e sem recursão nem crash.</t>
+  </si>
+  <si>
+    <t>19;20</t>
   </si>
 </sst>
 </file>
@@ -1574,7 +1613,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EC672E4-36B7-4DA7-B920-AB9B161145A3}">
-  <dimension ref="A1:L1011"/>
+  <dimension ref="A1:L1009"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.28515625" style="5" customWidth="1"/>
@@ -1588,7 +1627,8 @@
     <col min="9" max="9" width="8.7109375" style="7" customWidth="1"/>
     <col min="10" max="10" width="12.85546875" style="6" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="49" style="5" customWidth="1"/>
-    <col min="12" max="14" width="5.7109375" style="5" customWidth="1"/>
+    <col min="12" max="12" width="8.7109375" style="14" customWidth="1"/>
+    <col min="13" max="14" width="5.7109375" style="5" customWidth="1"/>
     <col min="15" max="27" width="8.7109375" style="5" customWidth="1"/>
     <col min="28" max="16384" width="14.42578125" style="5"/>
   </cols>
@@ -1663,7 +1703,7 @@
       <c r="K5" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="L5" s="12" t="s">
+      <c r="L5" s="3" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1701,7 +1741,7 @@
       <c r="K6" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="L6" s="17" t="s">
+      <c r="L6" s="15" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1739,7 +1779,7 @@
       <c r="K7" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="L7" s="17">
+      <c r="L7" s="15">
         <v>43</v>
       </c>
     </row>
@@ -1777,7 +1817,7 @@
       <c r="K8" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="L8" s="17" t="s">
+      <c r="L8" s="15" t="s">
         <v>36</v>
       </c>
     </row>
@@ -1815,7 +1855,7 @@
       <c r="K9" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="L9" s="17" t="s">
+      <c r="L9" s="15" t="s">
         <v>41</v>
       </c>
     </row>
@@ -1853,7 +1893,7 @@
       <c r="K10" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="L10" s="17" t="s">
+      <c r="L10" s="15" t="s">
         <v>48</v>
       </c>
     </row>
@@ -1891,7 +1931,7 @@
       <c r="K11" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="L11" s="17" t="s">
+      <c r="L11" s="15" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1929,7 +1969,7 @@
       <c r="K12" s="17" t="s">
         <v>58</v>
       </c>
-      <c r="L12" s="17" t="s">
+      <c r="L12" s="15" t="s">
         <v>59</v>
       </c>
     </row>
@@ -1967,7 +2007,7 @@
       <c r="K13" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="L13" s="17" t="s">
+      <c r="L13" s="15" t="s">
         <v>64</v>
       </c>
     </row>
@@ -2005,7 +2045,7 @@
       <c r="K14" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="L14" s="17" t="s">
+      <c r="L14" s="15" t="s">
         <v>71</v>
       </c>
     </row>
@@ -2043,7 +2083,7 @@
       <c r="K15" s="17" t="s">
         <v>76</v>
       </c>
-      <c r="L15" s="17">
+      <c r="L15" s="15">
         <v>44</v>
       </c>
     </row>
@@ -2081,7 +2121,7 @@
       <c r="K16" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="L16" s="17" t="s">
+      <c r="L16" s="15" t="s">
         <v>80</v>
       </c>
     </row>
@@ -2119,7 +2159,7 @@
       <c r="K17" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="L17" s="17">
+      <c r="L17" s="15">
         <v>44</v>
       </c>
     </row>
@@ -2157,7 +2197,7 @@
       <c r="K18" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="L18" s="17" t="s">
+      <c r="L18" s="15" t="s">
         <v>91</v>
       </c>
     </row>
@@ -2195,7 +2235,7 @@
       <c r="K19" s="17" t="s">
         <v>97</v>
       </c>
-      <c r="L19" s="17" t="s">
+      <c r="L19" s="15" t="s">
         <v>59</v>
       </c>
     </row>
@@ -2233,7 +2273,7 @@
       <c r="K20" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="L20" s="17">
+      <c r="L20" s="15">
         <v>44</v>
       </c>
     </row>
@@ -2271,7 +2311,7 @@
       <c r="K21" s="17" t="s">
         <v>108</v>
       </c>
-      <c r="L21" s="17">
+      <c r="L21" s="15">
         <v>46</v>
       </c>
     </row>
@@ -2309,7 +2349,7 @@
       <c r="K22" s="17" t="s">
         <v>114</v>
       </c>
-      <c r="L22" s="17" t="s">
+      <c r="L22" s="15" t="s">
         <v>115</v>
       </c>
     </row>
@@ -2317,7 +2357,7 @@
       <c r="H23" s="16"/>
       <c r="J23" s="16"/>
       <c r="K23" s="17"/>
-      <c r="L23" s="17"/>
+      <c r="L23" s="15"/>
     </row>
     <row r="24" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
@@ -2330,7 +2370,7 @@
       <c r="H24" s="16"/>
       <c r="J24" s="16"/>
       <c r="K24" s="17"/>
-      <c r="L24" s="17"/>
+      <c r="L24" s="15"/>
     </row>
     <row r="25" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
@@ -2366,7 +2406,7 @@
       <c r="K25" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="L25" s="12" t="s">
+      <c r="L25" s="3" t="s">
         <v>15</v>
       </c>
     </row>
@@ -2404,7 +2444,7 @@
       <c r="K26" s="17" t="s">
         <v>123</v>
       </c>
-      <c r="L26" s="17">
+      <c r="L26" s="15">
         <v>42</v>
       </c>
     </row>
@@ -2442,7 +2482,7 @@
       <c r="K27" s="17" t="s">
         <v>128</v>
       </c>
-      <c r="L27" s="17">
+      <c r="L27" s="15">
         <v>42</v>
       </c>
     </row>
@@ -2480,7 +2520,7 @@
       <c r="K28" s="17" t="s">
         <v>133</v>
       </c>
-      <c r="L28" s="17">
+      <c r="L28" s="15">
         <v>42</v>
       </c>
     </row>
@@ -2518,7 +2558,7 @@
       <c r="K29" s="17" t="s">
         <v>138</v>
       </c>
-      <c r="L29" s="17">
+      <c r="L29" s="15">
         <v>42</v>
       </c>
     </row>
@@ -2548,8 +2588,8 @@
         <v>46141</v>
       </c>
       <c r="J30" s="16"/>
-      <c r="K30" s="17"/>
-      <c r="L30" s="17"/>
+      <c r="K30" s="7"/>
+      <c r="L30" s="15"/>
     </row>
     <row r="31" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="13" t="s">
@@ -2577,8 +2617,8 @@
         <v>46141</v>
       </c>
       <c r="J31" s="16"/>
-      <c r="K31" s="17"/>
-      <c r="L31" s="17"/>
+      <c r="K31" s="7"/>
+      <c r="L31" s="15"/>
     </row>
     <row r="32" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="13" t="s">
@@ -2606,8 +2646,8 @@
         <v>46141</v>
       </c>
       <c r="J32" s="16"/>
-      <c r="K32" s="17"/>
-      <c r="L32" s="17"/>
+      <c r="K32" s="7"/>
+      <c r="L32" s="15"/>
     </row>
     <row r="33" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="13" t="s">
@@ -2635,8 +2675,8 @@
         <v>46141</v>
       </c>
       <c r="J33" s="16"/>
-      <c r="K33" s="17"/>
-      <c r="L33" s="17"/>
+      <c r="K33" s="7"/>
+      <c r="L33" s="15"/>
     </row>
     <row r="34" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="18" t="s">
@@ -2664,8 +2704,8 @@
         <v>46140</v>
       </c>
       <c r="J34" s="16"/>
-      <c r="K34" s="17"/>
-      <c r="L34" s="17"/>
+      <c r="K34" s="7"/>
+      <c r="L34" s="15"/>
     </row>
     <row r="35" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="18" t="s">
@@ -2693,8 +2733,8 @@
         <v>46140</v>
       </c>
       <c r="J35" s="16"/>
-      <c r="K35" s="17"/>
-      <c r="L35" s="17"/>
+      <c r="K35" s="7"/>
+      <c r="L35" s="15"/>
     </row>
     <row r="36" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="18" t="s">
@@ -2722,8 +2762,8 @@
         <v>46140</v>
       </c>
       <c r="J36" s="16"/>
-      <c r="K36" s="17"/>
-      <c r="L36" s="17"/>
+      <c r="K36" s="7"/>
+      <c r="L36" s="15"/>
     </row>
     <row r="37" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="18" t="s">
@@ -2751,8 +2791,8 @@
         <v>46140</v>
       </c>
       <c r="J37" s="16"/>
-      <c r="K37" s="17"/>
-      <c r="L37" s="17"/>
+      <c r="K37" s="7"/>
+      <c r="L37" s="15"/>
     </row>
     <row r="38" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="18" t="s">
@@ -2773,11 +2813,11 @@
       <c r="F38" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="G38" s="6" t="s">
-        <v>23</v>
+      <c r="G38" s="7" t="s">
+        <v>122</v>
       </c>
       <c r="H38" s="16">
-        <v>46140</v>
+        <v>46138</v>
       </c>
       <c r="I38" s="7" t="s">
         <v>122</v>
@@ -2788,7 +2828,7 @@
       <c r="K38" s="17" t="s">
         <v>173</v>
       </c>
-      <c r="L38" s="17">
+      <c r="L38" s="15">
         <v>42</v>
       </c>
     </row>
@@ -2818,8 +2858,8 @@
         <v>46140</v>
       </c>
       <c r="J39" s="16"/>
-      <c r="K39" s="17"/>
-      <c r="L39" s="17"/>
+      <c r="K39" s="7"/>
+      <c r="L39" s="15"/>
     </row>
     <row r="40" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="18" t="s">
@@ -2847,8 +2887,8 @@
         <v>46140</v>
       </c>
       <c r="J40" s="16"/>
-      <c r="K40" s="17"/>
-      <c r="L40" s="17"/>
+      <c r="K40" s="7"/>
+      <c r="L40" s="15"/>
     </row>
     <row r="41" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="18" t="s">
@@ -2876,8 +2916,8 @@
         <v>46140</v>
       </c>
       <c r="J41" s="16"/>
-      <c r="K41" s="17"/>
-      <c r="L41" s="17"/>
+      <c r="K41" s="7"/>
+      <c r="L41" s="15"/>
     </row>
     <row r="42" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="18" t="s">
@@ -2905,8 +2945,8 @@
         <v>46140</v>
       </c>
       <c r="J42" s="16"/>
-      <c r="K42" s="17"/>
-      <c r="L42" s="17"/>
+      <c r="K42" s="7"/>
+      <c r="L42" s="15"/>
     </row>
     <row r="43" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="18" t="s">
@@ -2934,8 +2974,8 @@
         <v>46140</v>
       </c>
       <c r="J43" s="16"/>
-      <c r="K43" s="17"/>
-      <c r="L43" s="17"/>
+      <c r="K43" s="7"/>
+      <c r="L43" s="15"/>
     </row>
     <row r="44" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="18" t="s">
@@ -2963,8 +3003,8 @@
         <v>46140</v>
       </c>
       <c r="J44" s="16"/>
-      <c r="K44" s="17"/>
-      <c r="L44" s="17"/>
+      <c r="K44" s="7"/>
+      <c r="L44" s="15"/>
     </row>
     <row r="45" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="18" t="s">
@@ -2992,8 +3032,8 @@
         <v>46140</v>
       </c>
       <c r="J45" s="16"/>
-      <c r="K45" s="17"/>
-      <c r="L45" s="17"/>
+      <c r="K45" s="7"/>
+      <c r="L45" s="15"/>
     </row>
     <row r="46" spans="1:12" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="18" t="s">
@@ -3021,14 +3061,14 @@
         <v>46142</v>
       </c>
       <c r="J46" s="16"/>
-      <c r="K46" s="17"/>
-      <c r="L46" s="17"/>
+      <c r="K46" s="7"/>
+      <c r="L46" s="15"/>
     </row>
     <row r="47" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="H47" s="16"/>
       <c r="J47" s="16"/>
       <c r="K47" s="17"/>
-      <c r="L47" s="17"/>
+      <c r="L47" s="15"/>
     </row>
     <row r="48" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
@@ -3041,7 +3081,7 @@
       <c r="H48" s="16"/>
       <c r="J48" s="16"/>
       <c r="K48" s="17"/>
-      <c r="L48" s="17"/>
+      <c r="L48" s="15"/>
     </row>
     <row r="49" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="12" t="s">
@@ -3077,7 +3117,7 @@
       <c r="K49" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="L49" s="12" t="s">
+      <c r="L49" s="3" t="s">
         <v>15</v>
       </c>
     </row>
@@ -3107,8 +3147,8 @@
         <v>46141</v>
       </c>
       <c r="J50" s="16"/>
-      <c r="K50" s="17"/>
-      <c r="L50" s="17"/>
+      <c r="K50" s="7"/>
+      <c r="L50" s="15"/>
     </row>
     <row r="51" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="13" t="s">
@@ -3136,15 +3176,15 @@
         <v>46141</v>
       </c>
       <c r="J51" s="16"/>
-      <c r="K51" s="17"/>
-      <c r="L51" s="17"/>
+      <c r="K51" s="7"/>
+      <c r="L51" s="15"/>
     </row>
     <row r="52" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="13" t="s">
+      <c r="A52" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="B52" s="13" t="s">
-        <v>17</v>
+      <c r="B52" s="5" t="s">
+        <v>66</v>
       </c>
       <c r="C52" s="5" t="s">
         <v>214</v>
@@ -3156,33 +3196,42 @@
         <v>216</v>
       </c>
       <c r="F52" s="5" t="s">
-        <v>143</v>
+        <v>121</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>22</v>
+        <v>69</v>
       </c>
       <c r="H52" s="16">
         <v>46141</v>
       </c>
-      <c r="J52" s="16"/>
-      <c r="K52" s="17"/>
-      <c r="L52" s="17"/>
+      <c r="I52" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="J52" s="16">
+        <v>46138</v>
+      </c>
+      <c r="K52" s="17" t="s">
+        <v>217</v>
+      </c>
+      <c r="L52" s="15">
+        <v>42</v>
+      </c>
     </row>
     <row r="53" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B53" s="5" t="s">
         <v>66</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D53" s="14" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E53" s="17" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F53" s="5" t="s">
         <v>121</v>
@@ -3194,16 +3243,16 @@
         <v>46141</v>
       </c>
       <c r="I53" s="7" t="s">
-        <v>122</v>
+        <v>23</v>
       </c>
       <c r="J53" s="16">
-        <v>46138</v>
-      </c>
-      <c r="K53" s="17" t="s">
-        <v>221</v>
-      </c>
-      <c r="L53" s="17">
-        <v>42</v>
+        <v>46143</v>
+      </c>
+      <c r="K53" s="7" t="s">
+        <v>350</v>
+      </c>
+      <c r="L53" s="15" t="s">
+        <v>351</v>
       </c>
     </row>
     <row r="54" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3231,16 +3280,25 @@
       <c r="H54" s="16">
         <v>46141</v>
       </c>
-      <c r="J54" s="16"/>
-      <c r="K54" s="17"/>
-      <c r="L54" s="17"/>
+      <c r="I54" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J54" s="16">
+        <v>46143</v>
+      </c>
+      <c r="K54" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="L54" s="15" t="s">
+        <v>353</v>
+      </c>
     </row>
     <row r="55" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
         <v>226</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>66</v>
+        <v>43</v>
       </c>
       <c r="C55" s="5" t="s">
         <v>227</v>
@@ -3252,17 +3310,17 @@
         <v>229</v>
       </c>
       <c r="F55" s="5" t="s">
-        <v>121</v>
+        <v>143</v>
       </c>
       <c r="G55" s="6" t="s">
-        <v>69</v>
+        <v>46</v>
       </c>
       <c r="H55" s="16">
         <v>46141</v>
       </c>
       <c r="J55" s="16"/>
-      <c r="K55" s="17"/>
-      <c r="L55" s="17"/>
+      <c r="K55" s="7"/>
+      <c r="L55" s="15"/>
     </row>
     <row r="56" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
@@ -3290,8 +3348,8 @@
         <v>46141</v>
       </c>
       <c r="J56" s="16"/>
-      <c r="K56" s="17"/>
-      <c r="L56" s="17"/>
+      <c r="K56" s="7"/>
+      <c r="L56" s="15"/>
     </row>
     <row r="57" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
@@ -3319,8 +3377,8 @@
         <v>46141</v>
       </c>
       <c r="J57" s="16"/>
-      <c r="K57" s="17"/>
-      <c r="L57" s="17"/>
+      <c r="K57" s="7"/>
+      <c r="L57" s="15"/>
     </row>
     <row r="58" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
@@ -3348,20 +3406,20 @@
         <v>46141</v>
       </c>
       <c r="J58" s="16"/>
-      <c r="K58" s="17"/>
-      <c r="L58" s="17"/>
+      <c r="K58" s="7"/>
+      <c r="L58" s="15"/>
     </row>
     <row r="59" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="5" t="s">
+      <c r="A59" s="18" t="s">
         <v>242</v>
       </c>
       <c r="B59" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="C59" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C59" s="17" t="s">
         <v>243</v>
       </c>
-      <c r="D59" s="14" t="s">
+      <c r="D59" s="15" t="s">
         <v>244</v>
       </c>
       <c r="E59" s="17" t="s">
@@ -3371,14 +3429,14 @@
         <v>143</v>
       </c>
       <c r="G59" s="6" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="H59" s="16">
-        <v>46141</v>
+        <v>46140</v>
       </c>
       <c r="J59" s="16"/>
-      <c r="K59" s="17"/>
-      <c r="L59" s="17"/>
+      <c r="K59" s="7"/>
+      <c r="L59" s="15"/>
     </row>
     <row r="60" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="18" t="s">
@@ -3406,8 +3464,8 @@
         <v>46140</v>
       </c>
       <c r="J60" s="16"/>
-      <c r="K60" s="17"/>
-      <c r="L60" s="17"/>
+      <c r="K60" s="7"/>
+      <c r="L60" s="15"/>
     </row>
     <row r="61" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="18" t="s">
@@ -3426,7 +3484,7 @@
         <v>253</v>
       </c>
       <c r="F61" s="5" t="s">
-        <v>143</v>
+        <v>121</v>
       </c>
       <c r="G61" s="6" t="s">
         <v>23</v>
@@ -3434,16 +3492,25 @@
       <c r="H61" s="16">
         <v>46140</v>
       </c>
-      <c r="J61" s="16"/>
-      <c r="K61" s="17"/>
-      <c r="L61" s="17"/>
+      <c r="I61" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J61" s="16">
+        <v>46143</v>
+      </c>
+      <c r="K61" s="7" t="s">
+        <v>354</v>
+      </c>
+      <c r="L61" s="15" t="s">
+        <v>355</v>
+      </c>
     </row>
     <row r="62" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="18" t="s">
         <v>254</v>
       </c>
       <c r="B62" s="5" t="s">
-        <v>66</v>
+        <v>17</v>
       </c>
       <c r="C62" s="17" t="s">
         <v>255</v>
@@ -3455,7 +3522,7 @@
         <v>257</v>
       </c>
       <c r="F62" s="5" t="s">
-        <v>121</v>
+        <v>143</v>
       </c>
       <c r="G62" s="6" t="s">
         <v>23</v>
@@ -3464,8 +3531,8 @@
         <v>46140</v>
       </c>
       <c r="J62" s="16"/>
-      <c r="K62" s="17"/>
-      <c r="L62" s="17"/>
+      <c r="K62" s="7"/>
+      <c r="L62" s="15"/>
     </row>
     <row r="63" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="18" t="s">
@@ -3493,97 +3560,97 @@
         <v>46140</v>
       </c>
       <c r="J63" s="16"/>
-      <c r="K63" s="17"/>
-      <c r="L63" s="17"/>
+      <c r="K63" s="7"/>
+      <c r="L63" s="15"/>
     </row>
     <row r="64" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="18" t="s">
+      <c r="K64" s="17"/>
+      <c r="L64" s="15"/>
+    </row>
+    <row r="65" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="B64" s="5" t="s">
+      <c r="B65" s="1"/>
+      <c r="C65" s="12"/>
+      <c r="D65" s="3"/>
+      <c r="E65" s="4"/>
+      <c r="K65" s="17"/>
+      <c r="L65" s="15"/>
+    </row>
+    <row r="66" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B66" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C66" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="D66" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="E66" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F66" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="G66" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="H66" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="I66" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="J66" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="K66" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="L66" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="13" t="s">
+        <v>263</v>
+      </c>
+      <c r="B67" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="C64" s="17" t="s">
-        <v>263</v>
-      </c>
-      <c r="D64" s="15" t="s">
+      <c r="C67" s="5" t="s">
         <v>264</v>
       </c>
-      <c r="E64" s="17" t="s">
+      <c r="D67" s="14" t="s">
         <v>265</v>
       </c>
-      <c r="F64" s="5" t="s">
+      <c r="E67" s="17" t="s">
+        <v>266</v>
+      </c>
+      <c r="F67" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="G64" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="H64" s="16">
-        <v>46140</v>
-      </c>
-      <c r="J64" s="16"/>
-      <c r="K64" s="17"/>
-      <c r="L64" s="17"/>
-    </row>
-    <row r="65" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="K65" s="17"/>
-      <c r="L65" s="17"/>
-    </row>
-    <row r="66" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="B66" s="1"/>
-      <c r="C66" s="12"/>
-      <c r="D66" s="3"/>
-      <c r="E66" s="4"/>
-      <c r="K66" s="17"/>
-      <c r="L66" s="17"/>
-    </row>
-    <row r="67" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="B67" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="C67" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="D67" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="E67" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="F67" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="G67" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="H67" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="I67" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J67" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="K67" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="L67" s="12" t="s">
-        <v>15</v>
-      </c>
+      <c r="G67" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H67" s="16">
+        <v>46141</v>
+      </c>
+      <c r="J67" s="16"/>
+      <c r="K67" s="7"/>
+      <c r="L67" s="15"/>
     </row>
     <row r="68" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="13" t="s">
+      <c r="A68" s="5" t="s">
         <v>267</v>
       </c>
-      <c r="B68" s="13" t="s">
-        <v>17</v>
+      <c r="B68" s="5" t="s">
+        <v>66</v>
       </c>
       <c r="C68" s="5" t="s">
         <v>268</v>
@@ -3595,24 +3662,33 @@
         <v>270</v>
       </c>
       <c r="F68" s="5" t="s">
-        <v>143</v>
+        <v>121</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>22</v>
+        <v>69</v>
       </c>
       <c r="H68" s="16">
         <v>46141</v>
       </c>
-      <c r="J68" s="16"/>
-      <c r="K68" s="17"/>
-      <c r="L68" s="17"/>
+      <c r="I68" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J68" s="16">
+        <v>46143</v>
+      </c>
+      <c r="K68" s="7" t="s">
+        <v>356</v>
+      </c>
+      <c r="L68" s="15" t="s">
+        <v>357</v>
+      </c>
     </row>
     <row r="69" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
         <v>271</v>
       </c>
       <c r="B69" s="5" t="s">
-        <v>66</v>
+        <v>43</v>
       </c>
       <c r="C69" s="5" t="s">
         <v>272</v>
@@ -3624,17 +3700,17 @@
         <v>274</v>
       </c>
       <c r="F69" s="5" t="s">
-        <v>121</v>
+        <v>143</v>
       </c>
       <c r="G69" s="6" t="s">
-        <v>69</v>
+        <v>46</v>
       </c>
       <c r="H69" s="16">
         <v>46141</v>
       </c>
       <c r="J69" s="16"/>
-      <c r="K69" s="17"/>
-      <c r="L69" s="17"/>
+      <c r="K69" s="7"/>
+      <c r="L69" s="15"/>
     </row>
     <row r="70" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="5" t="s">
@@ -3647,10 +3723,10 @@
         <v>276</v>
       </c>
       <c r="D70" s="14" t="s">
+        <v>273</v>
+      </c>
+      <c r="E70" s="17" t="s">
         <v>277</v>
-      </c>
-      <c r="E70" s="17" t="s">
-        <v>278</v>
       </c>
       <c r="F70" s="5" t="s">
         <v>143</v>
@@ -3662,21 +3738,21 @@
         <v>46141</v>
       </c>
       <c r="J70" s="16"/>
-      <c r="K70" s="17"/>
-      <c r="L70" s="17"/>
+      <c r="K70" s="7"/>
+      <c r="L70" s="15"/>
     </row>
     <row r="71" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="B71" s="5" t="s">
         <v>43</v>
       </c>
       <c r="C71" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="D71" s="14" t="s">
         <v>280</v>
-      </c>
-      <c r="D71" s="14" t="s">
-        <v>277</v>
       </c>
       <c r="E71" s="17" t="s">
         <v>281</v>
@@ -3691,53 +3767,53 @@
         <v>46141</v>
       </c>
       <c r="J71" s="16"/>
-      <c r="K71" s="17"/>
-      <c r="L71" s="17"/>
+      <c r="K71" s="7"/>
+      <c r="L71" s="15"/>
     </row>
     <row r="72" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="5" t="s">
+      <c r="A72" s="18" t="s">
         <v>282</v>
       </c>
       <c r="B72" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="C72" s="5" t="s">
         <v>283</v>
       </c>
-      <c r="D72" s="14" t="s">
+      <c r="C72" s="17" t="s">
         <v>284</v>
       </c>
+      <c r="D72" s="15" t="s">
+        <v>285</v>
+      </c>
       <c r="E72" s="17" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F72" s="5" t="s">
         <v>143</v>
       </c>
       <c r="G72" s="6" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="H72" s="16">
-        <v>46141</v>
+        <v>46140</v>
       </c>
       <c r="J72" s="16"/>
-      <c r="K72" s="17"/>
-      <c r="L72" s="17"/>
+      <c r="K72" s="7"/>
+      <c r="L72" s="15"/>
     </row>
     <row r="73" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="18" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C73" s="17" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D73" s="15" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E73" s="17" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F73" s="5" t="s">
         <v>143</v>
@@ -3749,15 +3825,15 @@
         <v>46140</v>
       </c>
       <c r="J73" s="16"/>
-      <c r="K73" s="17"/>
-      <c r="L73" s="17"/>
+      <c r="K73" s="7"/>
+      <c r="L73" s="15"/>
     </row>
     <row r="74" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="18" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B74" s="5" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="C74" s="17" t="s">
         <v>293</v>
@@ -3778,21 +3854,21 @@
         <v>46140</v>
       </c>
       <c r="J74" s="16"/>
-      <c r="K74" s="17"/>
-      <c r="L74" s="17"/>
+      <c r="K74" s="7"/>
+      <c r="L74" s="15"/>
     </row>
     <row r="75" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="18" t="s">
         <v>296</v>
       </c>
       <c r="B75" s="5" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="C75" s="17" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D75" s="15" t="s">
-        <v>298</v>
+        <v>244</v>
       </c>
       <c r="E75" s="17" t="s">
         <v>299</v>
@@ -3807,160 +3883,187 @@
         <v>46140</v>
       </c>
       <c r="J75" s="16"/>
-      <c r="K75" s="17"/>
-      <c r="L75" s="17"/>
+      <c r="K75" s="7"/>
+      <c r="L75" s="15"/>
     </row>
     <row r="76" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="18" t="s">
-        <v>300</v>
-      </c>
-      <c r="B76" s="5" t="s">
-        <v>301</v>
-      </c>
-      <c r="C76" s="17" t="s">
-        <v>302</v>
-      </c>
-      <c r="D76" s="15" t="s">
-        <v>248</v>
-      </c>
-      <c r="E76" s="17" t="s">
-        <v>303</v>
-      </c>
-      <c r="F76" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="G76" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="H76" s="16">
-        <v>46140</v>
-      </c>
+      <c r="H76" s="16"/>
       <c r="J76" s="16"/>
       <c r="K76" s="17"/>
-      <c r="L76" s="17"/>
+      <c r="L76" s="15"/>
     </row>
     <row r="77" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="H77" s="16"/>
-      <c r="J77" s="16"/>
+      <c r="A77" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="B77" s="1"/>
       <c r="K77" s="17"/>
-      <c r="L77" s="17"/>
+      <c r="L77" s="15"/>
     </row>
     <row r="78" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="1" t="s">
+      <c r="A78" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="B78" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="C78" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="D78" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="E78" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="F78" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="G78" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="H78" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="I78" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="J78" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="K78" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="L78" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="79" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A79" s="5" t="s">
+        <v>301</v>
+      </c>
+      <c r="B79" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C79" s="5" t="s">
+        <v>302</v>
+      </c>
+      <c r="D79" s="14" t="s">
+        <v>303</v>
+      </c>
+      <c r="E79" s="17" t="s">
         <v>304</v>
       </c>
-      <c r="B78" s="1"/>
-      <c r="K78" s="17"/>
-      <c r="L78" s="17"/>
-    </row>
-    <row r="79" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="B79" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="C79" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="D79" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="E79" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="F79" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="G79" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="H79" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="I79" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="J79" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="K79" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="L79" s="12" t="s">
-        <v>15</v>
+      <c r="F79" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="G79" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="H79" s="16">
+        <v>46141</v>
+      </c>
+      <c r="I79" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J79" s="16">
+        <v>46143</v>
+      </c>
+      <c r="K79" s="7" t="s">
+        <v>358</v>
+      </c>
+      <c r="L79" s="15">
+        <v>48</v>
       </c>
     </row>
     <row r="80" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A80" s="5" t="s">
+      <c r="A80" s="18" t="s">
         <v>305</v>
       </c>
       <c r="B80" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="C80" s="5" t="s">
         <v>306</v>
       </c>
-      <c r="D80" s="14" t="s">
+      <c r="C80" s="17" t="s">
         <v>307</v>
       </c>
+      <c r="D80" s="15" t="s">
+        <v>308</v>
+      </c>
       <c r="E80" s="17" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="F80" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="G80" s="6" t="s">
-        <v>69</v>
+      <c r="G80" s="7" t="s">
+        <v>122</v>
       </c>
       <c r="H80" s="16">
-        <v>46141</v>
-      </c>
-      <c r="J80" s="16"/>
-      <c r="K80" s="17"/>
-      <c r="L80" s="17"/>
+        <v>46138</v>
+      </c>
+      <c r="I80" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="J80" s="16">
+        <v>46138</v>
+      </c>
+      <c r="K80" s="17" t="s">
+        <v>310</v>
+      </c>
+      <c r="L80" s="15">
+        <v>42</v>
+      </c>
     </row>
     <row r="81" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="5" t="s">
-        <v>309</v>
+      <c r="A81" s="18" t="s">
+        <v>311</v>
       </c>
       <c r="B81" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="C81" s="5" t="s">
-        <v>310</v>
-      </c>
-      <c r="D81" s="14" t="s">
-        <v>311</v>
+        <v>306</v>
+      </c>
+      <c r="C81" s="17" t="s">
+        <v>312</v>
+      </c>
+      <c r="D81" s="15" t="s">
+        <v>313</v>
       </c>
       <c r="E81" s="17" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="F81" s="5" t="s">
         <v>121</v>
       </c>
       <c r="G81" s="6" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="H81" s="16">
-        <v>46141</v>
-      </c>
-      <c r="J81" s="16"/>
-      <c r="K81" s="17"/>
-      <c r="L81" s="17"/>
+        <v>46140</v>
+      </c>
+      <c r="I81" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J81" s="16">
+        <v>46143</v>
+      </c>
+      <c r="K81" s="7" t="s">
+        <v>359</v>
+      </c>
+      <c r="L81" s="15" t="s">
+        <v>360</v>
+      </c>
     </row>
     <row r="82" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="18" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B82" s="5" t="s">
-        <v>314</v>
+        <v>306</v>
       </c>
       <c r="C82" s="17" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D82" s="15" t="s">
-        <v>316</v>
+        <v>294</v>
       </c>
       <c r="E82" s="17" t="s">
         <v>317</v>
@@ -3975,33 +4078,33 @@
         <v>46140</v>
       </c>
       <c r="I82" s="7" t="s">
-        <v>122</v>
+        <v>23</v>
       </c>
       <c r="J82" s="16">
-        <v>46138</v>
-      </c>
-      <c r="K82" s="17" t="s">
-        <v>318</v>
-      </c>
-      <c r="L82" s="17">
-        <v>42</v>
+        <v>46143</v>
+      </c>
+      <c r="K82" s="7" t="s">
+        <v>361</v>
+      </c>
+      <c r="L82" s="15" t="s">
+        <v>362</v>
       </c>
     </row>
     <row r="83" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="18" t="s">
+        <v>318</v>
+      </c>
+      <c r="B83" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="C83" s="17" t="s">
         <v>319</v>
       </c>
-      <c r="B83" s="5" t="s">
-        <v>314</v>
-      </c>
-      <c r="C83" s="17" t="s">
+      <c r="D83" s="15" t="s">
         <v>320</v>
       </c>
-      <c r="D83" s="15" t="s">
+      <c r="E83" s="17" t="s">
         <v>321</v>
-      </c>
-      <c r="E83" s="17" t="s">
-        <v>322</v>
       </c>
       <c r="F83" s="5" t="s">
         <v>121</v>
@@ -4012,53 +4115,71 @@
       <c r="H83" s="16">
         <v>46140</v>
       </c>
-      <c r="J83" s="16"/>
-      <c r="K83" s="17"/>
-      <c r="L83" s="17"/>
+      <c r="I83" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J83" s="16">
+        <v>46143</v>
+      </c>
+      <c r="K83" s="7" t="s">
+        <v>363</v>
+      </c>
+      <c r="L83" s="15" t="s">
+        <v>364</v>
+      </c>
     </row>
     <row r="84" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="B84" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="C84" s="17" t="s">
         <v>323</v>
       </c>
-      <c r="B84" s="5" t="s">
-        <v>314</v>
-      </c>
-      <c r="C84" s="17" t="s">
+      <c r="D84" s="15">
+        <v>9</v>
+      </c>
+      <c r="E84" s="17" t="s">
         <v>324</v>
-      </c>
-      <c r="D84" s="15" t="s">
-        <v>298</v>
-      </c>
-      <c r="E84" s="17" t="s">
-        <v>325</v>
       </c>
       <c r="F84" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="G84" s="6" t="s">
-        <v>23</v>
+      <c r="G84" s="7" t="s">
+        <v>122</v>
       </c>
       <c r="H84" s="16">
-        <v>46140</v>
-      </c>
-      <c r="J84" s="16"/>
-      <c r="K84" s="17"/>
-      <c r="L84" s="17"/>
+        <v>46138</v>
+      </c>
+      <c r="I84" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="J84" s="16">
+        <v>46138</v>
+      </c>
+      <c r="K84" s="17" t="s">
+        <v>325</v>
+      </c>
+      <c r="L84" s="15">
+        <v>42</v>
+      </c>
     </row>
     <row r="85" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="18" t="s">
+      <c r="A85" s="5" t="s">
         <v>326</v>
       </c>
       <c r="B85" s="5" t="s">
-        <v>314</v>
-      </c>
-      <c r="C85" s="17" t="s">
+        <v>306</v>
+      </c>
+      <c r="C85" s="5" t="s">
         <v>327</v>
       </c>
-      <c r="D85" s="15" t="s">
+      <c r="D85" s="14" t="s">
         <v>328</v>
       </c>
-      <c r="E85" s="17" t="s">
+      <c r="E85" s="5" t="s">
         <v>329</v>
       </c>
       <c r="F85" s="5" t="s">
@@ -4068,27 +4189,36 @@
         <v>23</v>
       </c>
       <c r="H85" s="16">
-        <v>46140</v>
-      </c>
-      <c r="J85" s="16"/>
-      <c r="K85" s="17"/>
-      <c r="L85" s="17"/>
+        <v>46142</v>
+      </c>
+      <c r="I85" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="J85" s="16">
+        <v>46143</v>
+      </c>
+      <c r="K85" s="7" t="s">
+        <v>365</v>
+      </c>
+      <c r="L85" s="15" t="s">
+        <v>366</v>
+      </c>
     </row>
     <row r="86" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="18" t="s">
+      <c r="A86" s="5" t="s">
         <v>330</v>
       </c>
       <c r="B86" s="5" t="s">
-        <v>314</v>
-      </c>
-      <c r="C86" s="17" t="s">
+        <v>306</v>
+      </c>
+      <c r="C86" s="5" t="s">
         <v>331</v>
       </c>
-      <c r="D86" s="15">
-        <v>9</v>
-      </c>
-      <c r="E86" s="17" t="s">
+      <c r="D86" s="14" t="s">
         <v>332</v>
+      </c>
+      <c r="E86" s="5" t="s">
+        <v>333</v>
       </c>
       <c r="F86" s="5" t="s">
         <v>121</v>
@@ -4097,88 +4227,106 @@
         <v>23</v>
       </c>
       <c r="H86" s="16">
-        <v>46140</v>
+        <v>46142</v>
       </c>
       <c r="I86" s="7" t="s">
-        <v>122</v>
+        <v>23</v>
       </c>
       <c r="J86" s="16">
-        <v>46138</v>
-      </c>
-      <c r="K86" s="17" t="s">
-        <v>333</v>
-      </c>
-      <c r="L86" s="17">
-        <v>42</v>
+        <v>46143</v>
+      </c>
+      <c r="K86" s="7" t="s">
+        <v>367</v>
+      </c>
+      <c r="L86" s="15" t="s">
+        <v>368</v>
       </c>
     </row>
     <row r="87" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="5" t="s">
+      <c r="A87" s="18" t="s">
         <v>334</v>
       </c>
       <c r="B87" s="5" t="s">
-        <v>314</v>
-      </c>
-      <c r="C87" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="C87" s="17" t="s">
+        <v>175</v>
+      </c>
+      <c r="D87" s="15" t="s">
         <v>335</v>
       </c>
-      <c r="D87" s="14" t="s">
+      <c r="E87" s="17" t="s">
         <v>336</v>
-      </c>
-      <c r="E87" s="5" t="s">
-        <v>337</v>
       </c>
       <c r="F87" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="G87" s="6" t="s">
-        <v>23</v>
+      <c r="G87" s="7" t="s">
+        <v>122</v>
       </c>
       <c r="H87" s="16">
-        <v>46142</v>
-      </c>
-      <c r="J87" s="16"/>
-      <c r="K87" s="17"/>
-      <c r="L87" s="17"/>
+        <v>46138</v>
+      </c>
+      <c r="I87" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="J87" s="16">
+        <v>46138</v>
+      </c>
+      <c r="K87" s="17" t="s">
+        <v>337</v>
+      </c>
+      <c r="L87" s="15" t="s">
+        <v>338</v>
+      </c>
     </row>
     <row r="88" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A88" s="5" t="s">
-        <v>338</v>
+      <c r="A88" s="18" t="s">
+        <v>339</v>
       </c>
       <c r="B88" s="5" t="s">
-        <v>314</v>
-      </c>
-      <c r="C88" s="5" t="s">
-        <v>339</v>
-      </c>
-      <c r="D88" s="14" t="s">
-        <v>340</v>
-      </c>
-      <c r="E88" s="5" t="s">
-        <v>341</v>
+        <v>306</v>
+      </c>
+      <c r="C88" s="17" t="s">
+        <v>179</v>
+      </c>
+      <c r="D88" s="15" t="s">
+        <v>335</v>
+      </c>
+      <c r="E88" s="17" t="s">
+        <v>317</v>
       </c>
       <c r="F88" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="G88" s="6" t="s">
-        <v>23</v>
+      <c r="G88" s="7" t="s">
+        <v>122</v>
       </c>
       <c r="H88" s="16">
-        <v>46142</v>
-      </c>
-      <c r="J88" s="16"/>
-      <c r="K88" s="17"/>
-      <c r="L88" s="17"/>
+        <v>46138</v>
+      </c>
+      <c r="I88" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="J88" s="16">
+        <v>46138</v>
+      </c>
+      <c r="K88" s="17" t="s">
+        <v>340</v>
+      </c>
+      <c r="L88" s="15">
+        <v>42</v>
+      </c>
     </row>
     <row r="89" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="18" t="s">
+        <v>341</v>
+      </c>
+      <c r="B89" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="C89" s="17" t="s">
         <v>342</v>
-      </c>
-      <c r="B89" s="5" t="s">
-        <v>314</v>
-      </c>
-      <c r="C89" s="17" t="s">
-        <v>175</v>
       </c>
       <c r="D89" s="15" t="s">
         <v>343</v>
@@ -4189,11 +4337,11 @@
       <c r="F89" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="G89" s="6" t="s">
-        <v>23</v>
+      <c r="G89" s="7" t="s">
+        <v>122</v>
       </c>
       <c r="H89" s="16">
-        <v>46140</v>
+        <v>46138</v>
       </c>
       <c r="I89" s="7" t="s">
         <v>122</v>
@@ -4204,25 +4352,25 @@
       <c r="K89" s="17" t="s">
         <v>345</v>
       </c>
-      <c r="L89" s="17" t="s">
+      <c r="L89" s="15">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="90" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A90" s="5" t="s">
         <v>346</v>
       </c>
-    </row>
-    <row r="90" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A90" s="18" t="s">
+      <c r="B90" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="C90" s="5" t="s">
         <v>347</v>
       </c>
-      <c r="B90" s="5" t="s">
-        <v>314</v>
-      </c>
-      <c r="C90" s="17" t="s">
-        <v>179</v>
-      </c>
-      <c r="D90" s="15" t="s">
-        <v>343</v>
-      </c>
-      <c r="E90" s="17" t="s">
-        <v>325</v>
+      <c r="D90" s="14" t="s">
+        <v>348</v>
+      </c>
+      <c r="E90" s="5" t="s">
+        <v>349</v>
       </c>
       <c r="F90" s="5" t="s">
         <v>121</v>
@@ -4231,115 +4379,50 @@
         <v>23</v>
       </c>
       <c r="H90" s="16">
-        <v>46140</v>
+        <v>46142</v>
       </c>
       <c r="I90" s="7" t="s">
-        <v>122</v>
+        <v>23</v>
       </c>
       <c r="J90" s="16">
-        <v>46138</v>
-      </c>
-      <c r="K90" s="17" t="s">
-        <v>348</v>
-      </c>
-      <c r="L90" s="17">
-        <v>42</v>
+        <v>46143</v>
+      </c>
+      <c r="K90" s="7" t="s">
+        <v>369</v>
+      </c>
+      <c r="L90" s="15" t="s">
+        <v>370</v>
       </c>
     </row>
     <row r="91" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A91" s="18" t="s">
-        <v>349</v>
-      </c>
-      <c r="B91" s="5" t="s">
-        <v>314</v>
-      </c>
-      <c r="C91" s="17" t="s">
-        <v>350</v>
-      </c>
-      <c r="D91" s="15" t="s">
-        <v>351</v>
-      </c>
-      <c r="E91" s="17" t="s">
-        <v>352</v>
-      </c>
-      <c r="F91" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="G91" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="H91" s="16">
-        <v>46140</v>
-      </c>
-      <c r="I91" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="J91" s="16">
-        <v>46138</v>
-      </c>
-      <c r="K91" s="17" t="s">
-        <v>353</v>
-      </c>
-      <c r="L91" s="17">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="92" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A92" s="5" t="s">
-        <v>354</v>
-      </c>
-      <c r="B92" s="5" t="s">
-        <v>314</v>
-      </c>
-      <c r="C92" s="5" t="s">
-        <v>355</v>
-      </c>
-      <c r="D92" s="14" t="s">
-        <v>356</v>
-      </c>
-      <c r="E92" s="5" t="s">
-        <v>357</v>
-      </c>
-      <c r="F92" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="G92" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="H92" s="16">
-        <v>46142</v>
-      </c>
-      <c r="J92" s="16"/>
-      <c r="K92" s="17"/>
-      <c r="L92" s="17"/>
-    </row>
-    <row r="93" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93"/>
-      <c r="H93" s="16"/>
-      <c r="J93" s="16"/>
-    </row>
-    <row r="97" spans="8:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="H97" s="16"/>
-      <c r="J97" s="16"/>
-    </row>
-    <row r="98" spans="8:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="H98" s="16"/>
-      <c r="J98" s="16"/>
-    </row>
-    <row r="99" spans="8:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="100" spans="8:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="101" spans="8:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="102" spans="8:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="103" spans="8:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="104" spans="8:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="105" spans="8:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="106" spans="8:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="107" spans="8:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="108" spans="8:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="109" spans="8:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="110" spans="8:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="111" spans="8:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="112" spans="8:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="A91"/>
+      <c r="H91" s="16"/>
+      <c r="J91" s="16"/>
+    </row>
+    <row r="95" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H95" s="16"/>
+      <c r="J95" s="16"/>
+    </row>
+    <row r="96" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="H96" s="16"/>
+      <c r="J96" s="16"/>
+    </row>
+    <row r="97" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="98" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="99" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="100" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="101" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="102" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="103" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="104" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="105" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="106" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="107" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="108" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="109" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="110" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="111" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="112" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="113" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="114" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="115" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -5237,8 +5320,6 @@
     <row r="1007" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="1008" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="1009" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="1010" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="1011" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>